<commit_message>
Lambda 2024-01-29   oms  保宏 销售订单优化
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-tms/src/main/resources/excel/logisticsBill.xlsx
+++ b/erp-server/erp-server-tms/src/main/resources/excel/logisticsBill.xlsx
@@ -46,11 +46,68 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>{.salesPlatformName}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.shopName}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.sourceCode}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.outstockCode}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.toCountry}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.orderTime}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.deliveryTime}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.signTime}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.channelName}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.trackNo}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.transportDays}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.trackStatusName}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.trackContent}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.orderTypeName}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>发货时间</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>签收时间</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>物流渠道</t>
@@ -61,70 +118,15 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>运输天数(天)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>运输状态</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>轨迹描述(最新)</t>
-  </si>
-  <si>
-    <t>运输天数(天)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.salesPlatformName}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.shopName}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.sourceCode}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.outstockCode}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.toCountry}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.orderTime}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.deliveryTime}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.signTime}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.channelName}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.trackNo}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.transportDays}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.trackStatusName}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.trackContent}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.orderTypeName}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -132,7 +134,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -146,19 +148,6 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF666666"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF666666"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
@@ -181,15 +170,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -522,75 +505,75 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>